<commit_message>
Day 05 Full Data Load completed
</commit_message>
<xml_diff>
--- a/data/raw/companies.xlsx
+++ b/data/raw/companies.xlsx
@@ -399,18 +399,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L102"/>
   <cols>
-    <col min="1" max="1" width="47.50390625" customWidth="1"/>
-    <col min="2" max="2" width="47.50390625" customWidth="1"/>
-    <col min="3" max="3" width="47.50390625" customWidth="1"/>
-    <col min="4" max="4" width="47.50390625" customWidth="1"/>
-    <col min="5" max="5" width="47.50390625" customWidth="1"/>
-    <col min="6" max="6" width="47.50390625" customWidth="1"/>
-    <col min="7" max="7" width="47.50390625" customWidth="1"/>
-    <col min="8" max="8" width="47.50390625" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" customWidth="1"/>
-    <col min="12" max="12" width="19.50390625" customWidth="1"/>
+    <col min="1" max="1" width="50.00390625" customWidth="1"/>
+    <col min="2" max="2" width="50.00390625" customWidth="1"/>
+    <col min="3" max="3" width="50.00390625" customWidth="1"/>
+    <col min="4" max="4" width="50.00390625" customWidth="1"/>
+    <col min="5" max="5" width="50.00390625" customWidth="1"/>
+    <col min="6" max="6" width="50.00390625" customWidth="1"/>
+    <col min="7" max="7" width="50.00390625" customWidth="1"/>
+    <col min="8" max="8" width="50.00390625" customWidth="1"/>
+    <col min="9" max="9" width="18.1640625" customWidth="1"/>
+    <col min="10" max="10" width="18.1640625" customWidth="1"/>
+    <col min="11" max="11" width="25.00390625" customWidth="1"/>
+    <col min="12" max="12" width="23.6640625" customWidth="1"/>
     <col min="13" max="13" width="16.6640625" customWidth="1"/>
     <col min="14" max="14" width="16.6640625" customWidth="1"/>
     <col min="15" max="15" width="16.6640625" customWidth="1"/>
@@ -4035,68 +4035,9 @@
         <v>'TVS Motor Company Ltd (TVSM) is engaged in manufacturing two-wheelers and its accessories</v>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" t="str">
-        <v>ULTRACEMCO</v>
-      </c>
-      <c r="C95" t="str">
-        <v>UltraTech Cement</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="str">
-        <v>UNIONBANK</v>
-      </c>
-      <c r="C96" t="str">
-        <v>United Spirits</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="str">
-        <v>UNITDSPR</v>
-      </c>
-      <c r="C97" t="str">
-        <v>United Spirits</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <v>VBL</v>
-      </c>
-      <c r="C98" t="str">
-        <v>Varun Beverages</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="str">
-        <v>VEDL</v>
-      </c>
-      <c r="C99" t="str">
-        <v>Vedanta</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="str">
-        <v>WIPRO</v>
-      </c>
-      <c r="C100" t="str">
-        <v>Wipro</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="str">
-        <v>ZOMATO</v>
-      </c>
-      <c r="C101" t="str">
-        <v>Zomato</v>
-      </c>
-    </row>
     <row r="102">
-      <c r="A102" t="str">
-        <v>ZYDUSLIFE</v>
-      </c>
       <c r="C102" t="str">
-        <v>Zydus Lifesciences</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>